<commit_message>
Add XYZ inventory analysis
</commit_message>
<xml_diff>
--- a/02-inventory-abc-analysis/inventory_optimization.xlsx
+++ b/02-inventory-abc-analysis/inventory_optimization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\retail-excel-analytics\02-inventory-abc-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5EB453-3CEC-4B61-BEBE-5B87CD98C382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C47C2EC8-8E31-4756-A197-CD19B0F8FB44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13380" windowHeight="15165" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13380" windowHeight="15165" tabRatio="500" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,8 @@
     <sheet name="SKU Data" sheetId="3" r:id="rId3"/>
     <sheet name="Assumptions" sheetId="6" r:id="rId4"/>
     <sheet name="ABC Analysis" sheetId="4" r:id="rId5"/>
-    <sheet name="Reorder Point Model" sheetId="5" r:id="rId6"/>
+    <sheet name="XYZ Analysis" sheetId="7" r:id="rId6"/>
+    <sheet name="Reorder Point Model" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="135">
   <si>
     <t>Inventory ABC Analysis &amp; Reorder Point Model</t>
   </si>
@@ -421,6 +422,42 @@
   </si>
   <si>
     <t>Value Share Check</t>
+  </si>
+  <si>
+    <t>Coefficient of Variation</t>
+  </si>
+  <si>
+    <t>XYZ Class</t>
+  </si>
+  <si>
+    <t>XYZ Classification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X up to </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y up to </t>
+  </si>
+  <si>
+    <t>z = remainder</t>
+  </si>
+  <si>
+    <t>XYZ Summary</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>XYZ Validation</t>
   </si>
 </sst>
 </file>
@@ -608,7 +645,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -645,11 +682,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -662,14 +698,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2646,105 +2682,111 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
     </row>
     <row r="5" spans="2:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28" t="s">
+      <c r="C5" s="36"/>
+      <c r="D5" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28" t="s">
+      <c r="E5" s="36"/>
+      <c r="F5" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28" t="s">
+      <c r="G5" s="36"/>
+      <c r="H5" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="I5" s="28"/>
+      <c r="I5" s="36"/>
     </row>
     <row r="6" spans="2:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="31">
+      <c r="B6" s="30">
         <f>SUM('ABC Analysis'!D2:D21)</f>
         <v>276997</v>
       </c>
-      <c r="C6" s="31"/>
-      <c r="D6" s="32">
+      <c r="C6" s="30"/>
+      <c r="D6" s="31">
         <f>'ABC Analysis'!B26</f>
         <v>8</v>
       </c>
-      <c r="E6" s="32"/>
-      <c r="F6" s="33">
+      <c r="E6" s="31"/>
+      <c r="F6" s="32">
         <f>'ABC Analysis'!E26</f>
         <v>0</v>
       </c>
-      <c r="G6" s="33"/>
-      <c r="H6" s="32">
+      <c r="G6" s="32"/>
+      <c r="H6" s="31">
         <f>AVERAGE('Reorder Point Model'!I2:I21)</f>
         <v>54.60994241513383</v>
       </c>
-      <c r="I6" s="32"/>
+      <c r="I6" s="31"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34" t="s">
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="34"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+      <c r="J9" s="33"/>
     </row>
     <row r="10" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="29" t="str">
+      <c r="B10" s="28" t="str">
         <f>INDEX('ABC Analysis'!B2:B21,MATCH(1,'ABC Analysis'!E2:E21,0))</f>
         <v>Fitness Tracker Band</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="30" t="str">
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="29" t="str">
         <f>INDEX('Reorder Point Model'!B2:B21,MATCH(MAX('Reorder Point Model'!I2:I21),'Reorder Point Model'!I2:I21,0))</f>
         <v>Fitness Tracker Band</v>
       </c>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="F10:J10"/>
     <mergeCell ref="B6:C6"/>
@@ -2753,12 +2795,6 @@
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="F9:J9"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3530,7 +3566,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9869F81E-4192-476A-8613-1DD04D5D3BB6}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
@@ -3612,6 +3648,32 @@
       </c>
       <c r="H6">
         <v>1.28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="18">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>127</v>
+      </c>
+      <c r="B11" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -4347,12 +4409,12 @@
       </c>
     </row>
     <row r="24" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A24" s="35" t="s">
+      <c r="A24" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
     </row>
     <row r="25" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
@@ -4427,24 +4489,24 @@
       <c r="D29" s="22"/>
     </row>
     <row r="30" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A30" s="36" t="s">
+      <c r="A30" s="20" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A31" s="37" t="s">
+      <c r="A31" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="38" t="b">
+      <c r="B31" s="27" t="b">
         <f>SUM(B26:B28)=COUNTA(A2:A21)</f>
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A32" s="37" t="s">
+      <c r="A32" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="B32" s="38" t="b">
+      <c r="B32" s="27" t="b">
         <f>ROUND(SUM(D26:D28),4)=1</f>
         <v>1</v>
       </c>
@@ -4470,6 +4532,719 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC011802-3106-4502-B7BB-E91DA0D5242D}">
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>'SKU Data'!A2</f>
+        <v>ELE-403</v>
+      </c>
+      <c r="B2" t="str">
+        <f>'SKU Data'!B2</f>
+        <v>Fitness Tracker Band</v>
+      </c>
+      <c r="C2" t="str">
+        <f>'SKU Data'!C2</f>
+        <v>Electronics</v>
+      </c>
+      <c r="D2" s="14">
+        <f>'SKU Data'!G2</f>
+        <v>5.05</v>
+      </c>
+      <c r="E2" s="14">
+        <f>'SKU Data'!H2</f>
+        <v>1.31</v>
+      </c>
+      <c r="F2" s="22">
+        <f>IFERROR(E2/D2, 0)</f>
+        <v>0.25940594059405941</v>
+      </c>
+      <c r="G2" t="str">
+        <f>IF(F2&lt;=Assumptions!$B$10, "X", IF(F2&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f>'SKU Data'!A3</f>
+        <v>FTW-201</v>
+      </c>
+      <c r="B3" t="str">
+        <f>'SKU Data'!B3</f>
+        <v>Running Sneakers</v>
+      </c>
+      <c r="C3" t="str">
+        <f>'SKU Data'!C3</f>
+        <v>Footwear</v>
+      </c>
+      <c r="D3" s="14">
+        <f>'SKU Data'!G3</f>
+        <v>2.25</v>
+      </c>
+      <c r="E3" s="14">
+        <f>'SKU Data'!H3</f>
+        <v>0.77</v>
+      </c>
+      <c r="F3" s="22">
+        <f t="shared" ref="F3:F21" si="0">IFERROR(E3/D3, 0)</f>
+        <v>0.34222222222222221</v>
+      </c>
+      <c r="G3" t="str">
+        <f>IF(F3&lt;=Assumptions!$B$10, "X", IF(F3&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f>'SKU Data'!A4</f>
+        <v>ACC-302</v>
+      </c>
+      <c r="B4" t="str">
+        <f>'SKU Data'!B4</f>
+        <v>Aviator Sunglasses</v>
+      </c>
+      <c r="C4" t="str">
+        <f>'SKU Data'!C4</f>
+        <v>Accessories</v>
+      </c>
+      <c r="D4" s="14">
+        <f>'SKU Data'!G4</f>
+        <v>4.2</v>
+      </c>
+      <c r="E4" s="14">
+        <f>'SKU Data'!H4</f>
+        <v>1.43</v>
+      </c>
+      <c r="F4" s="22">
+        <f t="shared" si="0"/>
+        <v>0.34047619047619043</v>
+      </c>
+      <c r="G4" t="str">
+        <f>IF(F4&lt;=Assumptions!$B$10, "X", IF(F4&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <f>'SKU Data'!A5</f>
+        <v>FTW-202</v>
+      </c>
+      <c r="B5" t="str">
+        <f>'SKU Data'!B5</f>
+        <v>Canvas Low-Top</v>
+      </c>
+      <c r="C5" t="str">
+        <f>'SKU Data'!C5</f>
+        <v>Footwear</v>
+      </c>
+      <c r="D5" s="14">
+        <f>'SKU Data'!G5</f>
+        <v>2.6</v>
+      </c>
+      <c r="E5" s="14">
+        <f>'SKU Data'!H5</f>
+        <v>0.73</v>
+      </c>
+      <c r="F5" s="22">
+        <f t="shared" si="0"/>
+        <v>0.28076923076923077</v>
+      </c>
+      <c r="G5" t="str">
+        <f>IF(F5&lt;=Assumptions!$B$10, "X", IF(F5&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <f>'SKU Data'!A6</f>
+        <v>ELE-401</v>
+      </c>
+      <c r="B6" t="str">
+        <f>'SKU Data'!B6</f>
+        <v>Wireless Earbuds</v>
+      </c>
+      <c r="C6" t="str">
+        <f>'SKU Data'!C6</f>
+        <v>Electronics</v>
+      </c>
+      <c r="D6" s="14">
+        <f>'SKU Data'!G6</f>
+        <v>1.58</v>
+      </c>
+      <c r="E6" s="14">
+        <f>'SKU Data'!H6</f>
+        <v>0.79</v>
+      </c>
+      <c r="F6" s="22">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="G6" t="str">
+        <f>IF(F6&lt;=Assumptions!$B$10, "X", IF(F6&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <f>'SKU Data'!A7</f>
+        <v>FTW-203</v>
+      </c>
+      <c r="B7" t="str">
+        <f>'SKU Data'!B7</f>
+        <v>Leather Ankle Boot</v>
+      </c>
+      <c r="C7" t="str">
+        <f>'SKU Data'!C7</f>
+        <v>Footwear</v>
+      </c>
+      <c r="D7" s="14">
+        <f>'SKU Data'!G7</f>
+        <v>0.86</v>
+      </c>
+      <c r="E7" s="14">
+        <f>'SKU Data'!H7</f>
+        <v>0.38</v>
+      </c>
+      <c r="F7" s="22">
+        <f t="shared" si="0"/>
+        <v>0.44186046511627908</v>
+      </c>
+      <c r="G7" t="str">
+        <f>IF(F7&lt;=Assumptions!$B$10, "X", IF(F7&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <f>'SKU Data'!A8</f>
+        <v>HOM-503</v>
+      </c>
+      <c r="B8" t="str">
+        <f>'SKU Data'!B8</f>
+        <v>Cotton Throw Blanket</v>
+      </c>
+      <c r="C8" t="str">
+        <f>'SKU Data'!C8</f>
+        <v>Home Goods</v>
+      </c>
+      <c r="D8" s="14">
+        <f>'SKU Data'!G8</f>
+        <v>2.81</v>
+      </c>
+      <c r="E8" s="14">
+        <f>'SKU Data'!H8</f>
+        <v>1.52</v>
+      </c>
+      <c r="F8" s="22">
+        <f t="shared" si="0"/>
+        <v>0.54092526690391463</v>
+      </c>
+      <c r="G8" t="str">
+        <f>IF(F8&lt;=Assumptions!$B$10, "X", IF(F8&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <f>'SKU Data'!A9</f>
+        <v>ELE-402</v>
+      </c>
+      <c r="B9" t="str">
+        <f>'SKU Data'!B9</f>
+        <v>Bluetooth Speaker</v>
+      </c>
+      <c r="C9" t="str">
+        <f>'SKU Data'!C9</f>
+        <v>Electronics</v>
+      </c>
+      <c r="D9" s="14">
+        <f>'SKU Data'!G9</f>
+        <v>1.56</v>
+      </c>
+      <c r="E9" s="14">
+        <f>'SKU Data'!H9</f>
+        <v>0.69</v>
+      </c>
+      <c r="F9" s="22">
+        <f t="shared" si="0"/>
+        <v>0.44230769230769224</v>
+      </c>
+      <c r="G9" t="str">
+        <f>IF(F9&lt;=Assumptions!$B$10, "X", IF(F9&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="str">
+        <f>'SKU Data'!A10</f>
+        <v>APP-101</v>
+      </c>
+      <c r="B10" t="str">
+        <f>'SKU Data'!B10</f>
+        <v>Classic Denim Jacket</v>
+      </c>
+      <c r="C10" t="str">
+        <f>'SKU Data'!C10</f>
+        <v>Apparel</v>
+      </c>
+      <c r="D10" s="14">
+        <f>'SKU Data'!G10</f>
+        <v>0.92</v>
+      </c>
+      <c r="E10" s="14">
+        <f>'SKU Data'!H10</f>
+        <v>0.34</v>
+      </c>
+      <c r="F10" s="22">
+        <f t="shared" si="0"/>
+        <v>0.36956521739130438</v>
+      </c>
+      <c r="G10" t="str">
+        <f>IF(F10&lt;=Assumptions!$B$10, "X", IF(F10&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="str">
+        <f>'SKU Data'!A11</f>
+        <v>APP-103</v>
+      </c>
+      <c r="B11" t="str">
+        <f>'SKU Data'!B11</f>
+        <v>Fleece Pullover Hoodie</v>
+      </c>
+      <c r="C11" t="str">
+        <f>'SKU Data'!C11</f>
+        <v>Apparel</v>
+      </c>
+      <c r="D11" s="14">
+        <f>'SKU Data'!G11</f>
+        <v>1.17</v>
+      </c>
+      <c r="E11" s="14">
+        <f>'SKU Data'!H11</f>
+        <v>0.33</v>
+      </c>
+      <c r="F11" s="22">
+        <f t="shared" si="0"/>
+        <v>0.2820512820512821</v>
+      </c>
+      <c r="G11" t="str">
+        <f>IF(F11&lt;=Assumptions!$B$10, "X", IF(F11&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="str">
+        <f>'SKU Data'!A12</f>
+        <v>FTW-204</v>
+      </c>
+      <c r="B12" t="str">
+        <f>'SKU Data'!B12</f>
+        <v>Slide Sandals</v>
+      </c>
+      <c r="C12" t="str">
+        <f>'SKU Data'!C12</f>
+        <v>Footwear</v>
+      </c>
+      <c r="D12" s="14">
+        <f>'SKU Data'!G12</f>
+        <v>2.33</v>
+      </c>
+      <c r="E12" s="14">
+        <f>'SKU Data'!H12</f>
+        <v>1</v>
+      </c>
+      <c r="F12" s="22">
+        <f t="shared" si="0"/>
+        <v>0.42918454935622319</v>
+      </c>
+      <c r="G12" t="str">
+        <f>IF(F12&lt;=Assumptions!$B$10, "X", IF(F12&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="str">
+        <f>'SKU Data'!A13</f>
+        <v>HOM-504</v>
+      </c>
+      <c r="B13" t="str">
+        <f>'SKU Data'!B13</f>
+        <v>Bamboo Cutting Board</v>
+      </c>
+      <c r="C13" t="str">
+        <f>'SKU Data'!C13</f>
+        <v>Home Goods</v>
+      </c>
+      <c r="D13" s="14">
+        <f>'SKU Data'!G13</f>
+        <v>2.06</v>
+      </c>
+      <c r="E13" s="14">
+        <f>'SKU Data'!H13</f>
+        <v>0.52</v>
+      </c>
+      <c r="F13" s="22">
+        <f t="shared" si="0"/>
+        <v>0.25242718446601942</v>
+      </c>
+      <c r="G13" t="str">
+        <f>IF(F13&lt;=Assumptions!$B$10, "X", IF(F13&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="str">
+        <f>'SKU Data'!A14</f>
+        <v>HOM-501</v>
+      </c>
+      <c r="B14" t="str">
+        <f>'SKU Data'!B14</f>
+        <v>Ceramic Coffee Mug Set</v>
+      </c>
+      <c r="C14" t="str">
+        <f>'SKU Data'!C14</f>
+        <v>Home Goods</v>
+      </c>
+      <c r="D14" s="14">
+        <f>'SKU Data'!G14</f>
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="E14" s="14">
+        <f>'SKU Data'!H14</f>
+        <v>0.61</v>
+      </c>
+      <c r="F14" s="22">
+        <f t="shared" si="0"/>
+        <v>0.26991150442477879</v>
+      </c>
+      <c r="G14" t="str">
+        <f>IF(F14&lt;=Assumptions!$B$10, "X", IF(F14&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="str">
+        <f>'SKU Data'!A15</f>
+        <v>APP-104</v>
+      </c>
+      <c r="B15" t="str">
+        <f>'SKU Data'!B15</f>
+        <v>Slim Fit Chinos</v>
+      </c>
+      <c r="C15" t="str">
+        <f>'SKU Data'!C15</f>
+        <v>Apparel</v>
+      </c>
+      <c r="D15" s="14">
+        <f>'SKU Data'!G15</f>
+        <v>0.67</v>
+      </c>
+      <c r="E15" s="14">
+        <f>'SKU Data'!H15</f>
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="F15" s="22">
+        <f t="shared" si="0"/>
+        <v>0.41791044776119407</v>
+      </c>
+      <c r="G15" t="str">
+        <f>IF(F15&lt;=Assumptions!$B$10, "X", IF(F15&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="str">
+        <f>'SKU Data'!A16</f>
+        <v>ACC-304</v>
+      </c>
+      <c r="B16" t="str">
+        <f>'SKU Data'!B16</f>
+        <v>Wool Beanie</v>
+      </c>
+      <c r="C16" t="str">
+        <f>'SKU Data'!C16</f>
+        <v>Accessories</v>
+      </c>
+      <c r="D16" s="14">
+        <f>'SKU Data'!G16</f>
+        <v>2.19</v>
+      </c>
+      <c r="E16" s="14">
+        <f>'SKU Data'!H16</f>
+        <v>0.77</v>
+      </c>
+      <c r="F16" s="22">
+        <f t="shared" si="0"/>
+        <v>0.35159817351598177</v>
+      </c>
+      <c r="G16" t="str">
+        <f>IF(F16&lt;=Assumptions!$B$10, "X", IF(F16&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="str">
+        <f>'SKU Data'!A17</f>
+        <v>ACC-301</v>
+      </c>
+      <c r="B17" t="str">
+        <f>'SKU Data'!B17</f>
+        <v>Leather Belt</v>
+      </c>
+      <c r="C17" t="str">
+        <f>'SKU Data'!C17</f>
+        <v>Accessories</v>
+      </c>
+      <c r="D17" s="14">
+        <f>'SKU Data'!G17</f>
+        <v>0.94</v>
+      </c>
+      <c r="E17" s="14">
+        <f>'SKU Data'!H17</f>
+        <v>0.25</v>
+      </c>
+      <c r="F17" s="22">
+        <f t="shared" si="0"/>
+        <v>0.26595744680851063</v>
+      </c>
+      <c r="G17" t="str">
+        <f>IF(F17&lt;=Assumptions!$B$10, "X", IF(F17&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="str">
+        <f>'SKU Data'!A18</f>
+        <v>ACC-303</v>
+      </c>
+      <c r="B18" t="str">
+        <f>'SKU Data'!B18</f>
+        <v>Canvas Tote Bag</v>
+      </c>
+      <c r="C18" t="str">
+        <f>'SKU Data'!C18</f>
+        <v>Accessories</v>
+      </c>
+      <c r="D18" s="14">
+        <f>'SKU Data'!G18</f>
+        <v>0.73</v>
+      </c>
+      <c r="E18" s="14">
+        <f>'SKU Data'!H18</f>
+        <v>0.39</v>
+      </c>
+      <c r="F18" s="22">
+        <f t="shared" si="0"/>
+        <v>0.53424657534246578</v>
+      </c>
+      <c r="G18" t="str">
+        <f>IF(F18&lt;=Assumptions!$B$10, "X", IF(F18&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="str">
+        <f>'SKU Data'!A19</f>
+        <v>ELE-404</v>
+      </c>
+      <c r="B19" t="str">
+        <f>'SKU Data'!B19</f>
+        <v>Phone Charging Cable</v>
+      </c>
+      <c r="C19" t="str">
+        <f>'SKU Data'!C19</f>
+        <v>Electronics</v>
+      </c>
+      <c r="D19" s="14">
+        <f>'SKU Data'!G19</f>
+        <v>1.51</v>
+      </c>
+      <c r="E19" s="14">
+        <f>'SKU Data'!H19</f>
+        <v>0.48</v>
+      </c>
+      <c r="F19" s="22">
+        <f t="shared" si="0"/>
+        <v>0.31788079470198677</v>
+      </c>
+      <c r="G19" t="str">
+        <f>IF(F19&lt;=Assumptions!$B$10, "X", IF(F19&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>X</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="str">
+        <f>'SKU Data'!A20</f>
+        <v>HOM-502</v>
+      </c>
+      <c r="B20" t="str">
+        <f>'SKU Data'!B20</f>
+        <v>Scented Candle</v>
+      </c>
+      <c r="C20" t="str">
+        <f>'SKU Data'!C20</f>
+        <v>Home Goods</v>
+      </c>
+      <c r="D20" s="14">
+        <f>'SKU Data'!G20</f>
+        <v>1.02</v>
+      </c>
+      <c r="E20" s="14">
+        <f>'SKU Data'!H20</f>
+        <v>0.52</v>
+      </c>
+      <c r="F20" s="22">
+        <f t="shared" si="0"/>
+        <v>0.50980392156862742</v>
+      </c>
+      <c r="G20" t="str">
+        <f>IF(F20&lt;=Assumptions!$B$10, "X", IF(F20&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="str">
+        <f>'SKU Data'!A21</f>
+        <v>APP-102</v>
+      </c>
+      <c r="B21" t="str">
+        <f>'SKU Data'!B21</f>
+        <v>Cotton Crew T-Shirt</v>
+      </c>
+      <c r="C21" t="str">
+        <f>'SKU Data'!C21</f>
+        <v>Apparel</v>
+      </c>
+      <c r="D21" s="14">
+        <f>'SKU Data'!G21</f>
+        <v>0.65</v>
+      </c>
+      <c r="E21" s="14">
+        <f>'SKU Data'!H21</f>
+        <v>0.34</v>
+      </c>
+      <c r="F21" s="22">
+        <f t="shared" si="0"/>
+        <v>0.52307692307692311</v>
+      </c>
+      <c r="G21" t="str">
+        <f>IF(F21&lt;=Assumptions!$B$10, "X", IF(F21&lt;=Assumptions!$B$11, "Y", "Z"))</f>
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A24" s="37" t="s">
+        <v>129</v>
+      </c>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="B25" s="23" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="B26" s="26">
+        <f>COUNTIF($G$2:$G$21,A26)</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="B27" s="26">
+        <f t="shared" ref="B27:B28" si="1">COUNTIF($G$2:$G$21,A27)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="B28">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="26">
+        <f>SUM(B26:B28)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="B31" s="37"/>
+    </row>
+    <row r="32" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A32" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" t="b">
+        <f>SUM(B26:B28)=COUNTA(A2:A21)</f>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A31:B31"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:O21"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Add ABC-XYZ inventory segmentation
</commit_message>
<xml_diff>
--- a/02-inventory-abc-analysis/inventory_optimization.xlsx
+++ b/02-inventory-abc-analysis/inventory_optimization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\retail-excel-analytics\02-inventory-abc-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C47C2EC8-8E31-4756-A197-CD19B0F8FB44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE26BA2-FC71-4C47-B5EB-8205D529C7E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13380" windowHeight="15165" tabRatio="500" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13380" windowHeight="15465" tabRatio="500" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,8 @@
     <sheet name="Assumptions" sheetId="6" r:id="rId4"/>
     <sheet name="ABC Analysis" sheetId="4" r:id="rId5"/>
     <sheet name="XYZ Analysis" sheetId="7" r:id="rId6"/>
-    <sheet name="Reorder Point Model" sheetId="5" r:id="rId7"/>
+    <sheet name="ABC-XYZ Matrix" sheetId="8" r:id="rId7"/>
+    <sheet name="Reorder Point Model" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="140">
   <si>
     <t>Inventory ABC Analysis &amp; Reorder Point Model</t>
   </si>
@@ -458,6 +459,21 @@
   </si>
   <si>
     <t>XYZ Validation</t>
+  </si>
+  <si>
+    <t>ABC Class</t>
+  </si>
+  <si>
+    <t>ABC-XYZ Segment</t>
+  </si>
+  <si>
+    <t>ABC-XYZ Matrix</t>
+  </si>
+  <si>
+    <t>ABC / XYZ</t>
+  </si>
+  <si>
+    <t>ABC-XYZ Validation</t>
   </si>
 </sst>
 </file>
@@ -472,7 +488,7 @@
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -602,6 +618,27 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -645,7 +682,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -686,6 +723,14 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -698,13 +743,22 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2682,111 +2736,105 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
-      <c r="J3" s="35"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
     </row>
     <row r="5" spans="2:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36" t="s">
+      <c r="C5" s="31"/>
+      <c r="D5" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36" t="s">
+      <c r="E5" s="31"/>
+      <c r="F5" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36" t="s">
+      <c r="G5" s="31"/>
+      <c r="H5" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="I5" s="36"/>
+      <c r="I5" s="31"/>
     </row>
     <row r="6" spans="2:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="30">
+      <c r="B6" s="34">
         <f>SUM('ABC Analysis'!D2:D21)</f>
         <v>276997</v>
       </c>
-      <c r="C6" s="30"/>
-      <c r="D6" s="31">
+      <c r="C6" s="34"/>
+      <c r="D6" s="35">
         <f>'ABC Analysis'!B26</f>
         <v>8</v>
       </c>
-      <c r="E6" s="31"/>
-      <c r="F6" s="32">
+      <c r="E6" s="35"/>
+      <c r="F6" s="36">
         <f>'ABC Analysis'!E26</f>
         <v>0</v>
       </c>
-      <c r="G6" s="32"/>
-      <c r="H6" s="31">
+      <c r="G6" s="36"/>
+      <c r="H6" s="35">
         <f>AVERAGE('Reorder Point Model'!I2:I21)</f>
         <v>54.60994241513383</v>
       </c>
-      <c r="I6" s="31"/>
+      <c r="I6" s="35"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="33" t="s">
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-      <c r="J9" s="33"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37"/>
     </row>
     <row r="10" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="28" t="str">
+      <c r="B10" s="32" t="str">
         <f>INDEX('ABC Analysis'!B2:B21,MATCH(1,'ABC Analysis'!E2:E21,0))</f>
         <v>Fitness Tracker Band</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="29" t="str">
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="33" t="str">
         <f>INDEX('Reorder Point Model'!B2:B21,MATCH(MAX('Reorder Point Model'!I2:I21),'Reorder Point Model'!I2:I21,0))</f>
         <v>Fitness Tracker Band</v>
       </c>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="F10:J10"/>
     <mergeCell ref="B6:C6"/>
@@ -2795,6 +2843,12 @@
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="F9:J9"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4409,12 +4463,12 @@
       </c>
     </row>
     <row r="24" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A24" s="37" t="s">
+      <c r="A24" s="38" t="s">
         <v>117</v>
       </c>
-      <c r="B24" s="37"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="37"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
     </row>
     <row r="25" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
@@ -4538,32 +4592,32 @@
   <cols>
     <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="39" t="s">
         <v>123</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="39" t="s">
         <v>124</v>
       </c>
     </row>
@@ -5168,12 +5222,12 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="18" x14ac:dyDescent="0.25">
-      <c r="A24" s="37" t="s">
+      <c r="A24" s="38" t="s">
         <v>129</v>
       </c>
-      <c r="B24" s="37"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="37"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
     </row>
     <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
@@ -5220,10 +5274,10 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="37" t="s">
+      <c r="A31" s="38" t="s">
         <v>134</v>
       </c>
-      <c r="B31" s="37"/>
+      <c r="B31" s="38"/>
     </row>
     <row r="32" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
@@ -5245,6 +5299,589 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3256B65B-FE07-414F-B43D-C164FE6ABD2B}">
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="39" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="39" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1" s="39" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>'SKU Data'!A2</f>
+        <v>ELE-403</v>
+      </c>
+      <c r="B2" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Fitness Tracker Band</v>
+      </c>
+      <c r="C2" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A2,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>A</v>
+      </c>
+      <c r="D2" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A2,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E2" t="str">
+        <f>C2&amp;D2</f>
+        <v>AX</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f>'SKU Data'!A3</f>
+        <v>FTW-201</v>
+      </c>
+      <c r="B3" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Running Sneakers</v>
+      </c>
+      <c r="C3" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A3,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>A</v>
+      </c>
+      <c r="D3" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A3,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E21" si="0">C3&amp;D3</f>
+        <v>AX</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f>'SKU Data'!A4</f>
+        <v>ACC-302</v>
+      </c>
+      <c r="B4" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Aviator Sunglasses</v>
+      </c>
+      <c r="C4" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A4,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>A</v>
+      </c>
+      <c r="D4" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A4,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="0"/>
+        <v>AX</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <f>'SKU Data'!A5</f>
+        <v>FTW-202</v>
+      </c>
+      <c r="B5" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Canvas Low-Top</v>
+      </c>
+      <c r="C5" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A5,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>A</v>
+      </c>
+      <c r="D5" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A5,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="0"/>
+        <v>AX</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <f>'SKU Data'!A6</f>
+        <v>ELE-401</v>
+      </c>
+      <c r="B6" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Wireless Earbuds</v>
+      </c>
+      <c r="C6" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A6,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>A</v>
+      </c>
+      <c r="D6" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A6,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="0"/>
+        <v>AX</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <f>'SKU Data'!A7</f>
+        <v>FTW-203</v>
+      </c>
+      <c r="B7" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Leather Ankle Boot</v>
+      </c>
+      <c r="C7" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A7,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>A</v>
+      </c>
+      <c r="D7" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A7,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E7" t="str">
+        <f t="shared" si="0"/>
+        <v>AX</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <f>'SKU Data'!A8</f>
+        <v>HOM-503</v>
+      </c>
+      <c r="B8" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Cotton Throw Blanket</v>
+      </c>
+      <c r="C8" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A8,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>A</v>
+      </c>
+      <c r="D8" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A8,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>Y</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" si="0"/>
+        <v>AY</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <f>'SKU Data'!A9</f>
+        <v>ELE-402</v>
+      </c>
+      <c r="B9" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Bluetooth Speaker</v>
+      </c>
+      <c r="C9" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A9,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>A</v>
+      </c>
+      <c r="D9" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A9,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="0"/>
+        <v>AX</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="str">
+        <f>'SKU Data'!A10</f>
+        <v>APP-101</v>
+      </c>
+      <c r="B10" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Classic Denim Jacket</v>
+      </c>
+      <c r="C10" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A10,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>B</v>
+      </c>
+      <c r="D10" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A10,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="0"/>
+        <v>BX</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="str">
+        <f>'SKU Data'!A11</f>
+        <v>APP-103</v>
+      </c>
+      <c r="B11" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Fleece Pullover Hoodie</v>
+      </c>
+      <c r="C11" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A11,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>B</v>
+      </c>
+      <c r="D11" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A11,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="0"/>
+        <v>BX</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="str">
+        <f>'SKU Data'!A12</f>
+        <v>FTW-204</v>
+      </c>
+      <c r="B12" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Slide Sandals</v>
+      </c>
+      <c r="C12" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A12,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>B</v>
+      </c>
+      <c r="D12" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A12,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="0"/>
+        <v>BX</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="str">
+        <f>'SKU Data'!A13</f>
+        <v>HOM-504</v>
+      </c>
+      <c r="B13" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Bamboo Cutting Board</v>
+      </c>
+      <c r="C13" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A13,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>B</v>
+      </c>
+      <c r="D13" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A13,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="0"/>
+        <v>BX</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="str">
+        <f>'SKU Data'!A14</f>
+        <v>HOM-501</v>
+      </c>
+      <c r="B14" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Ceramic Coffee Mug Set</v>
+      </c>
+      <c r="C14" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A14,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>B</v>
+      </c>
+      <c r="D14" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A14,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="0"/>
+        <v>BX</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="str">
+        <f>'SKU Data'!A15</f>
+        <v>APP-104</v>
+      </c>
+      <c r="B15" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Slim Fit Chinos</v>
+      </c>
+      <c r="C15" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A15,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>B</v>
+      </c>
+      <c r="D15" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A15,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="0"/>
+        <v>BX</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="str">
+        <f>'SKU Data'!A16</f>
+        <v>ACC-304</v>
+      </c>
+      <c r="B16" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Wool Beanie</v>
+      </c>
+      <c r="C16" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A16,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>C</v>
+      </c>
+      <c r="D16" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A16,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E16" t="str">
+        <f t="shared" si="0"/>
+        <v>CX</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="str">
+        <f>'SKU Data'!A17</f>
+        <v>ACC-301</v>
+      </c>
+      <c r="B17" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Leather Belt</v>
+      </c>
+      <c r="C17" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A17,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>C</v>
+      </c>
+      <c r="D17" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A17,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E17" t="str">
+        <f t="shared" si="0"/>
+        <v>CX</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="str">
+        <f>'SKU Data'!A18</f>
+        <v>ACC-303</v>
+      </c>
+      <c r="B18" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Canvas Tote Bag</v>
+      </c>
+      <c r="C18" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A18,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>C</v>
+      </c>
+      <c r="D18" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A18,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>Y</v>
+      </c>
+      <c r="E18" t="str">
+        <f t="shared" si="0"/>
+        <v>CY</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="str">
+        <f>'SKU Data'!A19</f>
+        <v>ELE-404</v>
+      </c>
+      <c r="B19" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Phone Charging Cable</v>
+      </c>
+      <c r="C19" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A19,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>C</v>
+      </c>
+      <c r="D19" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A19,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>X</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="0"/>
+        <v>CX</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="str">
+        <f>'SKU Data'!A20</f>
+        <v>HOM-502</v>
+      </c>
+      <c r="B20" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Scented Candle</v>
+      </c>
+      <c r="C20" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A20,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>C</v>
+      </c>
+      <c r="D20" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A20,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>Y</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" si="0"/>
+        <v>CY</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="str">
+        <f>'SKU Data'!A21</f>
+        <v>APP-102</v>
+      </c>
+      <c r="B21" t="str">
+        <f>SKUData[[#This Row],[Product]]</f>
+        <v>Cotton Crew T-Shirt</v>
+      </c>
+      <c r="C21" t="str">
+        <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A21,'ABC Analysis'!$A$2:$A$21,0))</f>
+        <v>C</v>
+      </c>
+      <c r="D21" t="str">
+        <f>INDEX('XYZ Analysis'!$G$2:$G$21,MATCH(A21,'XYZ Analysis'!$A$2:$A$21,0))</f>
+        <v>Y</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="0"/>
+        <v>CY</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A24" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="B24" s="41"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="41"/>
+    </row>
+    <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="39" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" s="42" t="s">
+        <v>130</v>
+      </c>
+      <c r="C25" s="43" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" s="43" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="43" t="s">
+        <v>95</v>
+      </c>
+      <c r="B26">
+        <f>COUNTIFS($C$2:$C$21, $A26, $D$2:$D$21, B$25)</f>
+        <v>7</v>
+      </c>
+      <c r="C26">
+        <f t="shared" ref="C26:D28" si="1">COUNTIFS($C$2:$C$21, $A26, $D$2:$D$21, C$25)</f>
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="43" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27">
+        <f t="shared" ref="B27:B28" si="2">COUNTIFS($C$2:$C$21, $A27, $D$2:$D$21, B$25)</f>
+        <v>6</v>
+      </c>
+      <c r="C27">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="43" t="s">
+        <v>97</v>
+      </c>
+      <c r="B28">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="C28">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="43" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29">
+        <f>SUM(B26:D28)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="A30" s="38"/>
+      <c r="B30" s="38"/>
+      <c r="C30" s="28"/>
+    </row>
+    <row r="31" spans="1:5" ht="18" x14ac:dyDescent="0.25">
+      <c r="A31" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="B31" s="38"/>
+      <c r="C31" s="38"/>
+    </row>
+    <row r="32" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="44" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" s="40" t="b">
+        <f>B29=COUNTA(A2:A21)</f>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A30:B30"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:O21"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Add policy-driven inventory replenishment
</commit_message>
<xml_diff>
--- a/02-inventory-abc-analysis/inventory_optimization.xlsx
+++ b/02-inventory-abc-analysis/inventory_optimization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\retail-excel-analytics\02-inventory-abc-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE26BA2-FC71-4C47-B5EB-8205D529C7E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F77DC1-EC6A-40B7-BE1C-2CA831B93EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13380" windowHeight="15465" tabRatio="500" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="15" windowWidth="14325" windowHeight="15465" tabRatio="500" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,8 @@
     <sheet name="ABC Analysis" sheetId="4" r:id="rId5"/>
     <sheet name="XYZ Analysis" sheetId="7" r:id="rId6"/>
     <sheet name="ABC-XYZ Matrix" sheetId="8" r:id="rId7"/>
-    <sheet name="Reorder Point Model" sheetId="5" r:id="rId8"/>
+    <sheet name="Inventory Policy" sheetId="9" r:id="rId8"/>
+    <sheet name="Reorder Point Model" sheetId="5" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -54,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="174">
   <si>
     <t>Inventory ABC Analysis &amp; Reorder Point Model</t>
   </si>
@@ -365,18 +366,6 @@
     <t>Annual Orders (EOQ)</t>
   </si>
   <si>
-    <t>Service Level by Class (Z-score)</t>
-  </si>
-  <si>
-    <t>~99% service level</t>
-  </si>
-  <si>
-    <t>~95% service level</t>
-  </si>
-  <si>
-    <t>~90% service level</t>
-  </si>
-  <si>
     <t>Inventory Optimization Assumptions</t>
   </si>
   <si>
@@ -474,6 +463,120 @@
   </si>
   <si>
     <t>ABC-XYZ Validation</t>
+  </si>
+  <si>
+    <t>Inventory Policy by ABC-XYZ Segment</t>
+  </si>
+  <si>
+    <t>Segment</t>
+  </si>
+  <si>
+    <t>Service Level</t>
+  </si>
+  <si>
+    <t>Review Frequency</t>
+  </si>
+  <si>
+    <t>Inventory Control</t>
+  </si>
+  <si>
+    <t>Business Action</t>
+  </si>
+  <si>
+    <t>AX</t>
+  </si>
+  <si>
+    <t>AY</t>
+  </si>
+  <si>
+    <t>AZ</t>
+  </si>
+  <si>
+    <t>BX</t>
+  </si>
+  <si>
+    <t>BY</t>
+  </si>
+  <si>
+    <t>BZ</t>
+  </si>
+  <si>
+    <t>CX</t>
+  </si>
+  <si>
+    <t>CY</t>
+  </si>
+  <si>
+    <t>CZ</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Very High</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>Prioritize replenishment</t>
+  </si>
+  <si>
+    <t>Monitor demand closely</t>
+  </si>
+  <si>
+    <t>Closely monitor uncertainty</t>
+  </si>
+  <si>
+    <t>Standard replenishment</t>
+  </si>
+  <si>
+    <t>Monitor variability</t>
+  </si>
+  <si>
+    <t>Review demand uncertainty</t>
+  </si>
+  <si>
+    <t>Simple replenishment</t>
+  </si>
+  <si>
+    <t>Policy Validation</t>
+  </si>
+  <si>
+    <t>Segment Count</t>
+  </si>
+  <si>
+    <t>Unique Segment Check</t>
+  </si>
+  <si>
+    <t>SKU-Level Inventory Policy</t>
+  </si>
+  <si>
+    <t>Policy Assignment Validation</t>
+  </si>
+  <si>
+    <t>Missing Policies</t>
+  </si>
+  <si>
+    <t>Policy Service Level Validation</t>
+  </si>
+  <si>
+    <t>Missing Z Scores</t>
+  </si>
+  <si>
+    <t>Missing Safety Stock</t>
+  </si>
+  <si>
+    <t>Missing Reorder Points</t>
   </si>
 </sst>
 </file>
@@ -488,7 +591,7 @@
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -639,6 +742,20 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -682,7 +799,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -726,11 +843,33 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="23" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -743,23 +882,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -890,7 +1030,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1800" b="1" strike="noStrike" spc="-1">
+              <a:rPr lang="en-US" sz="1800" b="1" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -1430,7 +1570,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike" spc="-1">
+                  <a:rPr lang="en-US" sz="1000" b="1" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
@@ -1543,7 +1683,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike" spc="-1">
+                  <a:rPr lang="en-US" sz="1000" b="1" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
@@ -1645,7 +1785,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1800" b="1" strike="noStrike" spc="-1">
+              <a:rPr lang="en-US" sz="1800" b="1" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -1979,7 +2119,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1800" b="1" strike="noStrike" spc="-1">
+              <a:rPr lang="en-US" sz="1800" b="1" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -2191,7 +2331,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike" spc="-1">
+                  <a:rPr lang="en-US" sz="1000" b="1" strike="noStrike" spc="-1">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
@@ -2736,105 +2876,111 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
     </row>
     <row r="5" spans="2:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31" t="s">
+      <c r="C5" s="48"/>
+      <c r="D5" s="48" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31" t="s">
+      <c r="E5" s="48"/>
+      <c r="F5" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31" t="s">
+      <c r="G5" s="48"/>
+      <c r="H5" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="I5" s="31"/>
+      <c r="I5" s="48"/>
     </row>
     <row r="6" spans="2:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="34">
+      <c r="B6" s="42">
         <f>SUM('ABC Analysis'!D2:D21)</f>
         <v>276997</v>
       </c>
-      <c r="C6" s="34"/>
-      <c r="D6" s="35">
+      <c r="C6" s="42"/>
+      <c r="D6" s="43">
         <f>'ABC Analysis'!B26</f>
         <v>8</v>
       </c>
-      <c r="E6" s="35"/>
-      <c r="F6" s="36">
+      <c r="E6" s="43"/>
+      <c r="F6" s="44">
         <f>'ABC Analysis'!E26</f>
         <v>0</v>
       </c>
-      <c r="G6" s="36"/>
-      <c r="H6" s="35">
-        <f>AVERAGE('Reorder Point Model'!I2:I21)</f>
+      <c r="G6" s="44"/>
+      <c r="H6" s="43">
+        <f>AVERAGE('Reorder Point Model'!J2:J21)</f>
         <v>54.60994241513383</v>
       </c>
-      <c r="I6" s="35"/>
+      <c r="I6" s="43"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37" t="s">
+      <c r="C9" s="45"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="37"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="45"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="45"/>
     </row>
     <row r="10" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="32" t="str">
+      <c r="B10" s="40" t="str">
         <f>INDEX('ABC Analysis'!B2:B21,MATCH(1,'ABC Analysis'!E2:E21,0))</f>
         <v>Fitness Tracker Band</v>
       </c>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="33" t="str">
-        <f>INDEX('Reorder Point Model'!B2:B21,MATCH(MAX('Reorder Point Model'!I2:I21),'Reorder Point Model'!I2:I21,0))</f>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="41" t="str">
+        <f>INDEX('Reorder Point Model'!B2:B21,MATCH(MAX('Reorder Point Model'!J2:J21),'Reorder Point Model'!J2:J21,0))</f>
         <v>Fitness Tracker Band</v>
       </c>
-      <c r="G10" s="33"/>
-      <c r="H10" s="33"/>
-      <c r="I10" s="33"/>
-      <c r="J10" s="33"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="F10:J10"/>
     <mergeCell ref="B6:C6"/>
@@ -2843,12 +2989,6 @@
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="F9:J9"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3625,40 +3765,41 @@
   <cols>
     <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="22"/>
     <col min="7" max="7" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="19" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="G3" s="20" t="s">
         <v>112</v>
-      </c>
-      <c r="G3" s="20" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B4" s="18">
         <v>0.8</v>
       </c>
       <c r="D4" t="s">
-        <v>113</v>
-      </c>
-      <c r="E4" s="18">
-        <v>0.99</v>
+        <v>109</v>
+      </c>
+      <c r="E4" s="22">
+        <v>99</v>
       </c>
       <c r="G4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H4">
         <v>2.33</v>
@@ -3666,19 +3807,19 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B5" s="18">
         <v>0.95</v>
       </c>
       <c r="D5" t="s">
-        <v>114</v>
-      </c>
-      <c r="E5" s="18">
-        <v>0.95</v>
+        <v>110</v>
+      </c>
+      <c r="E5" s="22">
+        <v>95</v>
       </c>
       <c r="G5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H5">
         <v>1.65</v>
@@ -3686,19 +3827,19 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B6" s="18">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>115</v>
-      </c>
-      <c r="E6" s="18">
-        <v>0.9</v>
+        <v>111</v>
+      </c>
+      <c r="E6" s="22">
+        <v>90</v>
       </c>
       <c r="G6" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H6">
         <v>1.28</v>
@@ -3706,12 +3847,12 @@
     </row>
     <row r="9" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="20" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B10" s="18">
         <v>0.5</v>
@@ -3719,7 +3860,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B11" s="18">
         <v>1</v>
@@ -3727,7 +3868,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -4463,25 +4604,25 @@
       </c>
     </row>
     <row r="24" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A24" s="38" t="s">
-        <v>117</v>
-      </c>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
+      <c r="A24" s="49" t="s">
+        <v>113</v>
+      </c>
+      <c r="B24" s="49"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
     </row>
     <row r="25" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
         <v>94</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C25" s="24" t="s">
         <v>90</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E25" s="21"/>
     </row>
@@ -4544,12 +4685,12 @@
     </row>
     <row r="30" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="20" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B31" s="27" t="b">
         <f>SUM(B26:B28)=COUNTA(A2:A21)</f>
@@ -4558,7 +4699,7 @@
     </row>
     <row r="32" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B32" s="27" t="b">
         <f>ROUND(SUM(D26:D28),4)=1</f>
@@ -4599,26 +4740,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="39" t="s">
+      <c r="C1" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="39" t="s">
+      <c r="D1" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="39" t="s">
+      <c r="E1" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="39" t="s">
-        <v>123</v>
-      </c>
-      <c r="G1" s="39" t="s">
-        <v>124</v>
+      <c r="F1" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" s="29" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -5222,24 +5363,24 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="18" x14ac:dyDescent="0.25">
-      <c r="A24" s="38" t="s">
-        <v>129</v>
-      </c>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
+      <c r="A24" s="49" t="s">
+        <v>125</v>
+      </c>
+      <c r="B24" s="49"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
     </row>
     <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
         <v>94</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="26" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B26" s="26">
         <f>COUNTIF($G$2:$G$21,A26)</f>
@@ -5248,7 +5389,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B27" s="26">
         <f t="shared" ref="B27:B28" si="1">COUNTIF($G$2:$G$21,A27)</f>
@@ -5257,7 +5398,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B28">
         <f t="shared" si="1"/>
@@ -5266,7 +5407,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="26" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B29" s="26">
         <f>SUM(B26:B28)</f>
@@ -5274,14 +5415,14 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="B31" s="38"/>
+      <c r="A31" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="B31" s="49"/>
     </row>
     <row r="32" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B32" t="b">
         <f>SUM(B26:B28)=COUNTA(A2:A21)</f>
@@ -5311,20 +5452,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="39" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="39" t="s">
-        <v>124</v>
-      </c>
-      <c r="E1" s="39" t="s">
-        <v>136</v>
+      <c r="C1" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="29" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -5768,29 +5909,29 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A24" s="41" t="s">
-        <v>137</v>
-      </c>
-      <c r="B24" s="41"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
+      <c r="A24" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" s="50"/>
+      <c r="C24" s="50"/>
+      <c r="D24" s="50"/>
     </row>
     <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="39" t="s">
-        <v>138</v>
-      </c>
-      <c r="B25" s="42" t="s">
-        <v>130</v>
-      </c>
-      <c r="C25" s="43" t="s">
-        <v>131</v>
-      </c>
-      <c r="D25" s="43" t="s">
-        <v>132</v>
+      <c r="A25" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="B25" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" s="32" t="s">
+        <v>127</v>
+      </c>
+      <c r="D25" s="32" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="43" t="s">
+      <c r="A26" s="32" t="s">
         <v>95</v>
       </c>
       <c r="B26">
@@ -5807,7 +5948,7 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="32" t="s">
         <v>96</v>
       </c>
       <c r="B27">
@@ -5824,7 +5965,7 @@
       </c>
     </row>
     <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="43" t="s">
+      <c r="A28" s="32" t="s">
         <v>97</v>
       </c>
       <c r="B28">
@@ -5841,8 +5982,8 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="43" t="s">
-        <v>133</v>
+      <c r="A29" s="32" t="s">
+        <v>129</v>
       </c>
       <c r="B29">
         <f>SUM(B26:D28)</f>
@@ -5850,22 +5991,22 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="A30" s="38"/>
-      <c r="B30" s="38"/>
+      <c r="A30" s="49"/>
+      <c r="B30" s="49"/>
       <c r="C30" s="28"/>
     </row>
     <row r="31" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="A31" s="38" t="s">
-        <v>139</v>
-      </c>
-      <c r="B31" s="38"/>
-      <c r="C31" s="38"/>
+      <c r="A31" s="49" t="s">
+        <v>135</v>
+      </c>
+      <c r="B31" s="49"/>
+      <c r="C31" s="49"/>
     </row>
     <row r="32" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="44" t="s">
-        <v>121</v>
-      </c>
-      <c r="B32" s="40" t="b">
+      <c r="A32" s="33" t="s">
+        <v>117</v>
+      </c>
+      <c r="B32" s="30" t="b">
         <f>B29=COUNTA(A2:A21)</f>
         <v>1</v>
       </c>
@@ -5882,27 +6023,982 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40362696-B0F6-4E0F-9B7A-74911454A646}">
+  <dimension ref="A1:H47"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" customWidth="1"/>
+    <col min="6" max="6" width="20.85546875" customWidth="1"/>
+    <col min="7" max="7" width="29.42578125" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="51" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+    </row>
+    <row r="3" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="36" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>131</v>
+      </c>
+      <c r="C3" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="E3" s="36" t="s">
+        <v>139</v>
+      </c>
+      <c r="F3" s="36" t="s">
+        <v>140</v>
+      </c>
+      <c r="G3" s="36" t="s">
+        <v>141</v>
+      </c>
+      <c r="H3" s="36"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D4" s="35">
+        <v>99</v>
+      </c>
+      <c r="E4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G4" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5">
+        <v>99</v>
+      </c>
+      <c r="E5" t="s">
+        <v>151</v>
+      </c>
+      <c r="F5" t="s">
+        <v>154</v>
+      </c>
+      <c r="G5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D6">
+        <v>99</v>
+      </c>
+      <c r="E6" t="s">
+        <v>151</v>
+      </c>
+      <c r="F6" t="s">
+        <v>154</v>
+      </c>
+      <c r="G6" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>145</v>
+      </c>
+      <c r="B7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D7">
+        <v>95</v>
+      </c>
+      <c r="E7" t="s">
+        <v>152</v>
+      </c>
+      <c r="F7" t="s">
+        <v>155</v>
+      </c>
+      <c r="G7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" t="s">
+        <v>127</v>
+      </c>
+      <c r="D8">
+        <v>95</v>
+      </c>
+      <c r="E8" t="s">
+        <v>152</v>
+      </c>
+      <c r="F8" t="s">
+        <v>155</v>
+      </c>
+      <c r="G8" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C9" t="s">
+        <v>128</v>
+      </c>
+      <c r="D9">
+        <v>95</v>
+      </c>
+      <c r="E9" t="s">
+        <v>152</v>
+      </c>
+      <c r="F9" t="s">
+        <v>155</v>
+      </c>
+      <c r="G9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B10" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D10">
+        <v>90</v>
+      </c>
+      <c r="E10" t="s">
+        <v>153</v>
+      </c>
+      <c r="F10" t="s">
+        <v>156</v>
+      </c>
+      <c r="G10" s="34" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D11">
+        <v>90</v>
+      </c>
+      <c r="E11" t="s">
+        <v>153</v>
+      </c>
+      <c r="F11" t="s">
+        <v>156</v>
+      </c>
+      <c r="G11" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C12" t="s">
+        <v>128</v>
+      </c>
+      <c r="D12">
+        <v>90</v>
+      </c>
+      <c r="E12" t="s">
+        <v>153</v>
+      </c>
+      <c r="F12" t="s">
+        <v>156</v>
+      </c>
+      <c r="G12" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A15" s="51" t="s">
+        <v>164</v>
+      </c>
+      <c r="B15" s="51"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="51"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="B16">
+        <f>COUNTA(A4:A12)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="B17" t="b">
+        <f>SUMPRODUCT((A4:A12&lt;&gt;"")/COUNTIF(A4:A12,A4:A12&amp;""))=9</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A20" s="51" t="s">
+        <v>167</v>
+      </c>
+      <c r="B20" s="51"/>
+      <c r="C20" s="51"/>
+      <c r="D20" s="51"/>
+      <c r="E20" s="51"/>
+    </row>
+    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D22" t="s">
+        <v>138</v>
+      </c>
+      <c r="E22" t="s">
+        <v>139</v>
+      </c>
+      <c r="F22" t="s">
+        <v>140</v>
+      </c>
+      <c r="G22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="str">
+        <f>'ABC-XYZ Matrix'!A2</f>
+        <v>ELE-403</v>
+      </c>
+      <c r="B23" t="str">
+        <f>'ABC-XYZ Matrix'!B2</f>
+        <v>Fitness Tracker Band</v>
+      </c>
+      <c r="C23" t="str">
+        <f>'ABC-XYZ Matrix'!E2</f>
+        <v>AX</v>
+      </c>
+      <c r="D23">
+        <f>IFERROR(INDEX($D$4:$D$12,MATCH(C23,$A$4:$A$12,0)),"Not Found")</f>
+        <v>99</v>
+      </c>
+      <c r="E23" t="str">
+        <f>IFERROR(INDEX($E$4:$E$12,MATCH(C23,$A$4:$A$12,0)),"Not Found")</f>
+        <v>Daily</v>
+      </c>
+      <c r="F23" t="str">
+        <f>IFERROR(INDEX($F$4:$F$12,MATCH(C23,$A$4:$A$12,0)),"Not Found")</f>
+        <v>Very High</v>
+      </c>
+      <c r="G23" t="str">
+        <f>IFERROR(INDEX($G$4:$G$12,MATCH(C23,$A$4:$A$12,0)),"Not Found")</f>
+        <v>Prioritize replenishment</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A3</f>
+        <v>FTW-201</v>
+      </c>
+      <c r="B24" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B3</f>
+        <v>Running Sneakers</v>
+      </c>
+      <c r="C24" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E3</f>
+        <v>AX</v>
+      </c>
+      <c r="D24">
+        <f t="shared" ref="D24:D42" si="0">IFERROR(INDEX($D$4:$D$12,MATCH(C24,$A$4:$A$12,0)),"Not Found")</f>
+        <v>99</v>
+      </c>
+      <c r="E24" t="str">
+        <f t="shared" ref="E24:E42" si="1">IFERROR(INDEX($E$4:$E$12,MATCH(C24,$A$4:$A$12,0)),"Not Found")</f>
+        <v>Daily</v>
+      </c>
+      <c r="F24" t="str">
+        <f t="shared" ref="F24:F42" si="2">IFERROR(INDEX($F$4:$F$12,MATCH(C24,$A$4:$A$12,0)),"Not Found")</f>
+        <v>Very High</v>
+      </c>
+      <c r="G24" t="str">
+        <f t="shared" ref="G24:G42" si="3">IFERROR(INDEX($G$4:$G$12,MATCH(C24,$A$4:$A$12,0)),"Not Found")</f>
+        <v>Prioritize replenishment</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="str">
+        <f>'ABC-XYZ Matrix'!A4</f>
+        <v>ACC-302</v>
+      </c>
+      <c r="B25" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B4</f>
+        <v>Aviator Sunglasses</v>
+      </c>
+      <c r="C25" t="str">
+        <f>'ABC-XYZ Matrix'!E4</f>
+        <v>AX</v>
+      </c>
+      <c r="D25">
+        <f t="shared" si="0"/>
+        <v>99</v>
+      </c>
+      <c r="E25" t="str">
+        <f t="shared" si="1"/>
+        <v>Daily</v>
+      </c>
+      <c r="F25" t="str">
+        <f t="shared" si="2"/>
+        <v>Very High</v>
+      </c>
+      <c r="G25" t="str">
+        <f t="shared" si="3"/>
+        <v>Prioritize replenishment</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A5</f>
+        <v>FTW-202</v>
+      </c>
+      <c r="B26" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B5</f>
+        <v>Canvas Low-Top</v>
+      </c>
+      <c r="C26" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E5</f>
+        <v>AX</v>
+      </c>
+      <c r="D26">
+        <f t="shared" si="0"/>
+        <v>99</v>
+      </c>
+      <c r="E26" t="str">
+        <f t="shared" si="1"/>
+        <v>Daily</v>
+      </c>
+      <c r="F26" t="str">
+        <f t="shared" si="2"/>
+        <v>Very High</v>
+      </c>
+      <c r="G26" t="str">
+        <f t="shared" si="3"/>
+        <v>Prioritize replenishment</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A6</f>
+        <v>ELE-401</v>
+      </c>
+      <c r="B27" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B6</f>
+        <v>Wireless Earbuds</v>
+      </c>
+      <c r="C27" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E6</f>
+        <v>AX</v>
+      </c>
+      <c r="D27">
+        <f t="shared" si="0"/>
+        <v>99</v>
+      </c>
+      <c r="E27" t="str">
+        <f t="shared" si="1"/>
+        <v>Daily</v>
+      </c>
+      <c r="F27" t="str">
+        <f t="shared" si="2"/>
+        <v>Very High</v>
+      </c>
+      <c r="G27" t="str">
+        <f t="shared" si="3"/>
+        <v>Prioritize replenishment</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A7</f>
+        <v>FTW-203</v>
+      </c>
+      <c r="B28" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B7</f>
+        <v>Leather Ankle Boot</v>
+      </c>
+      <c r="C28" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E7</f>
+        <v>AX</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="0"/>
+        <v>99</v>
+      </c>
+      <c r="E28" t="str">
+        <f t="shared" si="1"/>
+        <v>Daily</v>
+      </c>
+      <c r="F28" t="str">
+        <f t="shared" si="2"/>
+        <v>Very High</v>
+      </c>
+      <c r="G28" t="str">
+        <f t="shared" si="3"/>
+        <v>Prioritize replenishment</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A8</f>
+        <v>HOM-503</v>
+      </c>
+      <c r="B29" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B8</f>
+        <v>Cotton Throw Blanket</v>
+      </c>
+      <c r="C29" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E8</f>
+        <v>AY</v>
+      </c>
+      <c r="D29">
+        <f t="shared" si="0"/>
+        <v>99</v>
+      </c>
+      <c r="E29" t="str">
+        <f t="shared" si="1"/>
+        <v>Daily</v>
+      </c>
+      <c r="F29" t="str">
+        <f t="shared" si="2"/>
+        <v>Very High</v>
+      </c>
+      <c r="G29" t="str">
+        <f t="shared" si="3"/>
+        <v>Monitor demand closely</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A9</f>
+        <v>ELE-402</v>
+      </c>
+      <c r="B30" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B9</f>
+        <v>Bluetooth Speaker</v>
+      </c>
+      <c r="C30" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E9</f>
+        <v>AX</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="0"/>
+        <v>99</v>
+      </c>
+      <c r="E30" t="str">
+        <f t="shared" si="1"/>
+        <v>Daily</v>
+      </c>
+      <c r="F30" t="str">
+        <f t="shared" si="2"/>
+        <v>Very High</v>
+      </c>
+      <c r="G30" t="str">
+        <f t="shared" si="3"/>
+        <v>Prioritize replenishment</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A10</f>
+        <v>APP-101</v>
+      </c>
+      <c r="B31" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B10</f>
+        <v>Classic Denim Jacket</v>
+      </c>
+      <c r="C31" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E10</f>
+        <v>BX</v>
+      </c>
+      <c r="D31">
+        <f t="shared" si="0"/>
+        <v>95</v>
+      </c>
+      <c r="E31" t="str">
+        <f t="shared" si="1"/>
+        <v>Weekly</v>
+      </c>
+      <c r="F31" t="str">
+        <f t="shared" si="2"/>
+        <v>High</v>
+      </c>
+      <c r="G31" t="str">
+        <f t="shared" si="3"/>
+        <v>Standard replenishment</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A11</f>
+        <v>APP-103</v>
+      </c>
+      <c r="B32" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B11</f>
+        <v>Fleece Pullover Hoodie</v>
+      </c>
+      <c r="C32" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E11</f>
+        <v>BX</v>
+      </c>
+      <c r="D32">
+        <f t="shared" si="0"/>
+        <v>95</v>
+      </c>
+      <c r="E32" t="str">
+        <f t="shared" si="1"/>
+        <v>Weekly</v>
+      </c>
+      <c r="F32" t="str">
+        <f t="shared" si="2"/>
+        <v>High</v>
+      </c>
+      <c r="G32" t="str">
+        <f t="shared" si="3"/>
+        <v>Standard replenishment</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A12</f>
+        <v>FTW-204</v>
+      </c>
+      <c r="B33" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B12</f>
+        <v>Slide Sandals</v>
+      </c>
+      <c r="C33" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E12</f>
+        <v>BX</v>
+      </c>
+      <c r="D33">
+        <f t="shared" si="0"/>
+        <v>95</v>
+      </c>
+      <c r="E33" t="str">
+        <f t="shared" si="1"/>
+        <v>Weekly</v>
+      </c>
+      <c r="F33" t="str">
+        <f t="shared" si="2"/>
+        <v>High</v>
+      </c>
+      <c r="G33" t="str">
+        <f t="shared" si="3"/>
+        <v>Standard replenishment</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A13</f>
+        <v>HOM-504</v>
+      </c>
+      <c r="B34" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B13</f>
+        <v>Bamboo Cutting Board</v>
+      </c>
+      <c r="C34" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E13</f>
+        <v>BX</v>
+      </c>
+      <c r="D34">
+        <f t="shared" si="0"/>
+        <v>95</v>
+      </c>
+      <c r="E34" t="str">
+        <f t="shared" si="1"/>
+        <v>Weekly</v>
+      </c>
+      <c r="F34" t="str">
+        <f t="shared" si="2"/>
+        <v>High</v>
+      </c>
+      <c r="G34" t="str">
+        <f t="shared" si="3"/>
+        <v>Standard replenishment</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A14</f>
+        <v>HOM-501</v>
+      </c>
+      <c r="B35" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B14</f>
+        <v>Ceramic Coffee Mug Set</v>
+      </c>
+      <c r="C35" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E14</f>
+        <v>BX</v>
+      </c>
+      <c r="D35">
+        <f t="shared" si="0"/>
+        <v>95</v>
+      </c>
+      <c r="E35" t="str">
+        <f t="shared" si="1"/>
+        <v>Weekly</v>
+      </c>
+      <c r="F35" t="str">
+        <f t="shared" si="2"/>
+        <v>High</v>
+      </c>
+      <c r="G35" t="str">
+        <f t="shared" si="3"/>
+        <v>Standard replenishment</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A15</f>
+        <v>APP-104</v>
+      </c>
+      <c r="B36" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B15</f>
+        <v>Slim Fit Chinos</v>
+      </c>
+      <c r="C36" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E15</f>
+        <v>BX</v>
+      </c>
+      <c r="D36">
+        <f t="shared" si="0"/>
+        <v>95</v>
+      </c>
+      <c r="E36" t="str">
+        <f t="shared" si="1"/>
+        <v>Weekly</v>
+      </c>
+      <c r="F36" t="str">
+        <f t="shared" si="2"/>
+        <v>High</v>
+      </c>
+      <c r="G36" t="str">
+        <f t="shared" si="3"/>
+        <v>Standard replenishment</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A16</f>
+        <v>ACC-304</v>
+      </c>
+      <c r="B37" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B16</f>
+        <v>Wool Beanie</v>
+      </c>
+      <c r="C37" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E16</f>
+        <v>CX</v>
+      </c>
+      <c r="D37">
+        <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="E37" t="str">
+        <f t="shared" si="1"/>
+        <v>Monthly</v>
+      </c>
+      <c r="F37" t="str">
+        <f t="shared" si="2"/>
+        <v>Standard</v>
+      </c>
+      <c r="G37" t="str">
+        <f t="shared" si="3"/>
+        <v>Simple replenishment</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A17</f>
+        <v>ACC-301</v>
+      </c>
+      <c r="B38" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B17</f>
+        <v>Leather Belt</v>
+      </c>
+      <c r="C38" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E17</f>
+        <v>CX</v>
+      </c>
+      <c r="D38">
+        <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="E38" t="str">
+        <f t="shared" si="1"/>
+        <v>Monthly</v>
+      </c>
+      <c r="F38" t="str">
+        <f t="shared" si="2"/>
+        <v>Standard</v>
+      </c>
+      <c r="G38" t="str">
+        <f t="shared" si="3"/>
+        <v>Simple replenishment</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A18</f>
+        <v>ACC-303</v>
+      </c>
+      <c r="B39" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B18</f>
+        <v>Canvas Tote Bag</v>
+      </c>
+      <c r="C39" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E18</f>
+        <v>CY</v>
+      </c>
+      <c r="D39">
+        <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="E39" t="str">
+        <f t="shared" si="1"/>
+        <v>Monthly</v>
+      </c>
+      <c r="F39" t="str">
+        <f t="shared" si="2"/>
+        <v>Standard</v>
+      </c>
+      <c r="G39" t="str">
+        <f t="shared" si="3"/>
+        <v>Monitor variability</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A19</f>
+        <v>ELE-404</v>
+      </c>
+      <c r="B40" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B19</f>
+        <v>Phone Charging Cable</v>
+      </c>
+      <c r="C40" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E19</f>
+        <v>CX</v>
+      </c>
+      <c r="D40">
+        <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="E40" t="str">
+        <f t="shared" si="1"/>
+        <v>Monthly</v>
+      </c>
+      <c r="F40" t="str">
+        <f t="shared" si="2"/>
+        <v>Standard</v>
+      </c>
+      <c r="G40" t="str">
+        <f t="shared" si="3"/>
+        <v>Simple replenishment</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A20</f>
+        <v>HOM-502</v>
+      </c>
+      <c r="B41" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B20</f>
+        <v>Scented Candle</v>
+      </c>
+      <c r="C41" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E20</f>
+        <v>CY</v>
+      </c>
+      <c r="D41">
+        <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="E41" t="str">
+        <f t="shared" si="1"/>
+        <v>Monthly</v>
+      </c>
+      <c r="F41" t="str">
+        <f t="shared" si="2"/>
+        <v>Standard</v>
+      </c>
+      <c r="G41" t="str">
+        <f t="shared" si="3"/>
+        <v>Monitor variability</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!A21</f>
+        <v>APP-102</v>
+      </c>
+      <c r="B42" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!B21</f>
+        <v>Cotton Crew T-Shirt</v>
+      </c>
+      <c r="C42" s="5" t="str">
+        <f>'ABC-XYZ Matrix'!E21</f>
+        <v>CY</v>
+      </c>
+      <c r="D42">
+        <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="E42" t="str">
+        <f t="shared" si="1"/>
+        <v>Monthly</v>
+      </c>
+      <c r="F42" t="str">
+        <f t="shared" si="2"/>
+        <v>Standard</v>
+      </c>
+      <c r="G42" t="str">
+        <f t="shared" si="3"/>
+        <v>Monitor variability</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A45" s="52" t="s">
+        <v>168</v>
+      </c>
+      <c r="B45" s="52"/>
+      <c r="C45" s="52"/>
+      <c r="D45" s="52"/>
+    </row>
+    <row r="46" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A46" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="B46" s="29">
+        <f>COUNTA(A23:A42)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A47" s="29" t="s">
+        <v>169</v>
+      </c>
+      <c r="B47">
+        <f>COUNTIF(D23:D42,"Not Found")</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A45:D45"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="13" max="13" width="8" customWidth="1"/>
-    <col min="14" max="14" width="10" customWidth="1"/>
-    <col min="15" max="15" width="20" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="10" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="13" max="13" width="9.140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8" customWidth="1"/>
+    <col min="15" max="15" width="10" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>34</v>
       </c>
@@ -5912,35 +7008,39 @@
       <c r="C1" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="I1" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M1" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>'SKU Data'!A2</f>
         <v>ELE-403</v>
@@ -5953,49 +7053,50 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A2,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>A</v>
       </c>
-      <c r="D2" s="14">
+      <c r="D2" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A2,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>AX</v>
+      </c>
+      <c r="E2" s="14">
         <f>'SKU Data'!G2</f>
         <v>5.05</v>
       </c>
-      <c r="E2" s="14">
+      <c r="F2" s="14">
         <f>'SKU Data'!H2</f>
         <v>1.31</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>'SKU Data'!I2</f>
         <v>45</v>
       </c>
-      <c r="G2" s="14">
-        <f t="shared" ref="G2:G21" si="0">INDEX($N$2:$N$4,MATCH(C2,$M$2:$M$4,0))</f>
+      <c r="H2" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M2,Assumptions!$E$4:$E$6,0))</f>
         <v>2.33</v>
       </c>
-      <c r="H2" s="15">
-        <f t="shared" ref="H2:H21" si="1">G2*E2*SQRT(F2)</f>
+      <c r="I2" s="15">
+        <f t="shared" ref="I2:I21" si="0">H2*F2*SQRT(G2)</f>
         <v>20.475450863167826</v>
       </c>
-      <c r="I2" s="15">
-        <f t="shared" ref="I2:I21" si="2">(D2*F2)+H2</f>
+      <c r="J2" s="15">
+        <f t="shared" ref="J2:J21" si="1">(E2*G2)+I2</f>
         <v>247.72545086316782</v>
       </c>
-      <c r="J2" s="15">
+      <c r="K2" s="15">
         <f>SQRT((2*'SKU Data'!F2*'SKU Data'!J2)/('SKU Data'!D2*'SKU Data'!K2))</f>
         <v>173.82524957929544</v>
       </c>
-      <c r="K2" s="16">
-        <f>IFERROR('SKU Data'!F2/J2,0)</f>
+      <c r="L2" s="16">
+        <f>IFERROR('SKU Data'!F2/K2,0)</f>
         <v>10.614108160151668</v>
       </c>
-      <c r="M2" t="s">
-        <v>95</v>
-      </c>
-      <c r="N2" s="9">
-        <v>2.33</v>
-      </c>
-      <c r="O2" s="17" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M2" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D2,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>99</v>
+      </c>
+      <c r="O2" s="9"/>
+      <c r="P2" s="17"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f>'SKU Data'!A3</f>
         <v>FTW-201</v>
@@ -6008,49 +7109,50 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A3,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>A</v>
       </c>
-      <c r="D3" s="14">
+      <c r="D3" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A3,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>AX</v>
+      </c>
+      <c r="E3" s="14">
         <f>'SKU Data'!G3</f>
         <v>2.25</v>
       </c>
-      <c r="E3" s="14">
+      <c r="F3" s="14">
         <f>'SKU Data'!H3</f>
         <v>0.77</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <f>'SKU Data'!I3</f>
         <v>14</v>
       </c>
-      <c r="G3" s="14">
-        <f t="shared" si="0"/>
+      <c r="H3" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M3,Assumptions!$E$4:$E$6,0))</f>
         <v>2.33</v>
       </c>
-      <c r="H3" s="15">
+      <c r="I3" s="15">
+        <f t="shared" si="0"/>
+        <v>6.7129075176111286</v>
+      </c>
+      <c r="J3" s="15">
         <f t="shared" si="1"/>
-        <v>6.7129075176111286</v>
-      </c>
-      <c r="I3" s="15">
-        <f t="shared" si="2"/>
         <v>38.212907517611129</v>
       </c>
-      <c r="J3" s="15">
+      <c r="K3" s="15">
         <f>SQRT((2*'SKU Data'!F3*'SKU Data'!J3)/('SKU Data'!D3*'SKU Data'!K3))</f>
         <v>139.78202443113702</v>
       </c>
-      <c r="K3" s="16">
-        <f>IFERROR('SKU Data'!F3/J3,0)</f>
+      <c r="L3" s="16">
+        <f>IFERROR('SKU Data'!F3/K3,0)</f>
         <v>5.873430459611507</v>
       </c>
-      <c r="M3" t="s">
-        <v>96</v>
-      </c>
-      <c r="N3" s="9">
-        <v>1.65</v>
-      </c>
-      <c r="O3" s="17" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M3" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D3,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>99</v>
+      </c>
+      <c r="O3" s="9"/>
+      <c r="P3" s="17"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f>'SKU Data'!A4</f>
         <v>ACC-302</v>
@@ -6063,49 +7165,50 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A4,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>A</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A4,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>AX</v>
+      </c>
+      <c r="E4" s="14">
         <f>'SKU Data'!G4</f>
         <v>4.2</v>
       </c>
-      <c r="E4" s="14">
+      <c r="F4" s="14">
         <f>'SKU Data'!H4</f>
         <v>1.43</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <f>'SKU Data'!I4</f>
         <v>10</v>
       </c>
-      <c r="G4" s="14">
-        <f t="shared" si="0"/>
+      <c r="H4" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M4,Assumptions!$E$4:$E$6,0))</f>
         <v>2.33</v>
       </c>
-      <c r="H4" s="15">
+      <c r="I4" s="15">
+        <f t="shared" si="0"/>
+        <v>10.536392935915025</v>
+      </c>
+      <c r="J4" s="15">
         <f t="shared" si="1"/>
-        <v>10.536392935915025</v>
-      </c>
-      <c r="I4" s="15">
-        <f t="shared" si="2"/>
         <v>52.536392935915025</v>
       </c>
-      <c r="J4" s="15">
+      <c r="K4" s="15">
         <f>SQRT((2*'SKU Data'!F4*'SKU Data'!J4)/('SKU Data'!D4*'SKU Data'!K4))</f>
         <v>232.71394457573874</v>
       </c>
-      <c r="K4" s="16">
-        <f>IFERROR('SKU Data'!F4/J4,0)</f>
+      <c r="L4" s="16">
+        <f>IFERROR('SKU Data'!F4/K4,0)</f>
         <v>6.587486636414571</v>
       </c>
-      <c r="M4" t="s">
-        <v>97</v>
-      </c>
-      <c r="N4" s="9">
-        <v>1.28</v>
-      </c>
-      <c r="O4" s="17" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M4" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D4,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>99</v>
+      </c>
+      <c r="O4" s="9"/>
+      <c r="P4" s="17"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f>'SKU Data'!A5</f>
         <v>FTW-202</v>
@@ -6118,40 +7221,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A5,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>A</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A5,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>AX</v>
+      </c>
+      <c r="E5" s="14">
         <f>'SKU Data'!G5</f>
         <v>2.6</v>
       </c>
-      <c r="E5" s="14">
+      <c r="F5" s="14">
         <f>'SKU Data'!H5</f>
         <v>0.73</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <f>'SKU Data'!I5</f>
         <v>14</v>
       </c>
-      <c r="G5" s="14">
-        <f t="shared" si="0"/>
+      <c r="H5" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M5,Assumptions!$E$4:$E$6,0))</f>
         <v>2.33</v>
       </c>
-      <c r="H5" s="15">
+      <c r="I5" s="15">
+        <f t="shared" si="0"/>
+        <v>6.3641850491637975</v>
+      </c>
+      <c r="J5" s="15">
         <f t="shared" si="1"/>
-        <v>6.3641850491637975</v>
-      </c>
-      <c r="I5" s="15">
-        <f t="shared" si="2"/>
         <v>42.7641850491638</v>
       </c>
-      <c r="J5" s="15">
+      <c r="K5" s="15">
         <f>SQRT((2*'SKU Data'!F5*'SKU Data'!J5)/('SKU Data'!D5*'SKU Data'!K5))</f>
         <v>178.18070500579921</v>
       </c>
-      <c r="K5" s="16">
-        <f>IFERROR('SKU Data'!F5/J5,0)</f>
+      <c r="L5" s="16">
+        <f>IFERROR('SKU Data'!F5/K5,0)</f>
         <v>5.3260536822385625</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M5" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D5,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f>'SKU Data'!A6</f>
         <v>ELE-401</v>
@@ -6164,40 +7275,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A6,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>A</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A6,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>AX</v>
+      </c>
+      <c r="E6" s="14">
         <f>'SKU Data'!G6</f>
         <v>1.58</v>
       </c>
-      <c r="E6" s="14">
+      <c r="F6" s="14">
         <f>'SKU Data'!H6</f>
         <v>0.79</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <f>'SKU Data'!I6</f>
         <v>21</v>
       </c>
-      <c r="G6" s="14">
-        <f t="shared" si="0"/>
+      <c r="H6" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M6,Assumptions!$E$4:$E$6,0))</f>
         <v>2.33</v>
       </c>
-      <c r="H6" s="15">
+      <c r="I6" s="15">
+        <f t="shared" si="0"/>
+        <v>8.4351470817052157</v>
+      </c>
+      <c r="J6" s="15">
         <f t="shared" si="1"/>
-        <v>8.4351470817052157</v>
-      </c>
-      <c r="I6" s="15">
-        <f t="shared" si="2"/>
         <v>41.615147081705217</v>
       </c>
-      <c r="J6" s="15">
+      <c r="K6" s="15">
         <f>SQRT((2*'SKU Data'!F6*'SKU Data'!J6)/('SKU Data'!D6*'SKU Data'!K6))</f>
         <v>113.95975596846527</v>
       </c>
-      <c r="K6" s="16">
-        <f>IFERROR('SKU Data'!F6/J6,0)</f>
+      <c r="L6" s="16">
+        <f>IFERROR('SKU Data'!F6/K6,0)</f>
         <v>5.0456408502586907</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M6" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D6,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f>'SKU Data'!A7</f>
         <v>FTW-203</v>
@@ -6210,40 +7329,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A7,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>A</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A7,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>AX</v>
+      </c>
+      <c r="E7" s="14">
         <f>'SKU Data'!G7</f>
         <v>0.86</v>
       </c>
-      <c r="E7" s="14">
+      <c r="F7" s="14">
         <f>'SKU Data'!H7</f>
         <v>0.38</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <f>'SKU Data'!I7</f>
         <v>45</v>
       </c>
-      <c r="G7" s="14">
-        <f t="shared" si="0"/>
+      <c r="H7" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M7,Assumptions!$E$4:$E$6,0))</f>
         <v>2.33</v>
       </c>
-      <c r="H7" s="15">
+      <c r="I7" s="15">
+        <f t="shared" si="0"/>
+        <v>5.9394437618349425</v>
+      </c>
+      <c r="J7" s="15">
         <f t="shared" si="1"/>
-        <v>5.9394437618349425</v>
-      </c>
-      <c r="I7" s="15">
-        <f t="shared" si="2"/>
         <v>44.639443761834947</v>
       </c>
-      <c r="J7" s="15">
+      <c r="K7" s="15">
         <f>SQRT((2*'SKU Data'!F7*'SKU Data'!J7)/('SKU Data'!D7*'SKU Data'!K7))</f>
         <v>81.137652673211349</v>
       </c>
-      <c r="K7" s="16">
-        <f>IFERROR('SKU Data'!F7/J7,0)</f>
+      <c r="L7" s="16">
+        <f>IFERROR('SKU Data'!F7/K7,0)</f>
         <v>3.8576417937629222</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M7" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D7,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f>'SKU Data'!A8</f>
         <v>HOM-503</v>
@@ -6256,40 +7383,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A8,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>A</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A8,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>AY</v>
+      </c>
+      <c r="E8" s="14">
         <f>'SKU Data'!G8</f>
         <v>2.81</v>
       </c>
-      <c r="E8" s="14">
+      <c r="F8" s="14">
         <f>'SKU Data'!H8</f>
         <v>1.52</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <f>'SKU Data'!I8</f>
         <v>14</v>
       </c>
-      <c r="G8" s="14">
-        <f t="shared" si="0"/>
+      <c r="H8" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M8,Assumptions!$E$4:$E$6,0))</f>
         <v>2.33</v>
       </c>
-      <c r="H8" s="15">
+      <c r="I8" s="15">
+        <f t="shared" si="0"/>
+        <v>13.251453800998592</v>
+      </c>
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
-        <v>13.251453800998592</v>
-      </c>
-      <c r="I8" s="15">
-        <f t="shared" si="2"/>
         <v>52.591453800998593</v>
       </c>
-      <c r="J8" s="15">
+      <c r="K8" s="15">
         <f>SQRT((2*'SKU Data'!F8*'SKU Data'!J8)/('SKU Data'!D8*'SKU Data'!K8))</f>
         <v>198.64071418854024</v>
       </c>
-      <c r="K8" s="16">
-        <f>IFERROR('SKU Data'!F8/J8,0)</f>
+      <c r="L8" s="16">
+        <f>IFERROR('SKU Data'!F8/K8,0)</f>
         <v>5.1550358353427397</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M8" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D8,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f>'SKU Data'!A9</f>
         <v>ELE-402</v>
@@ -6302,40 +7437,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A9,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>A</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A9,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>AX</v>
+      </c>
+      <c r="E9" s="14">
         <f>'SKU Data'!G9</f>
         <v>1.56</v>
       </c>
-      <c r="E9" s="14">
+      <c r="F9" s="14">
         <f>'SKU Data'!H9</f>
         <v>0.69</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <f>'SKU Data'!I9</f>
         <v>45</v>
       </c>
-      <c r="G9" s="14">
-        <f t="shared" si="0"/>
+      <c r="H9" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M9,Assumptions!$E$4:$E$6,0))</f>
         <v>2.33</v>
       </c>
-      <c r="H9" s="15">
+      <c r="I9" s="15">
+        <f t="shared" si="0"/>
+        <v>10.784779462279236</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v>10.784779462279236</v>
-      </c>
-      <c r="I9" s="15">
-        <f t="shared" si="2"/>
         <v>80.984779462279235</v>
       </c>
-      <c r="J9" s="15">
+      <c r="K9" s="15">
         <f>SQRT((2*'SKU Data'!F9*'SKU Data'!J9)/('SKU Data'!D9*'SKU Data'!K9))</f>
         <v>130.2529750140088</v>
       </c>
-      <c r="K9" s="16">
-        <f>IFERROR('SKU Data'!F9/J9,0)</f>
+      <c r="L9" s="16">
+        <f>IFERROR('SKU Data'!F9/K9,0)</f>
         <v>4.3837770303410615</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M9" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D9,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f>'SKU Data'!A10</f>
         <v>APP-101</v>
@@ -6348,40 +7491,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A10,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>B</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A10,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>BX</v>
+      </c>
+      <c r="E10" s="14">
         <f>'SKU Data'!G10</f>
         <v>0.92</v>
       </c>
-      <c r="E10" s="14">
+      <c r="F10" s="14">
         <f>'SKU Data'!H10</f>
         <v>0.34</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <f>'SKU Data'!I10</f>
         <v>7</v>
       </c>
-      <c r="G10" s="14">
-        <f t="shared" si="0"/>
+      <c r="H10" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M10,Assumptions!$E$4:$E$6,0))</f>
         <v>1.65</v>
       </c>
-      <c r="H10" s="15">
+      <c r="I10" s="15">
+        <f t="shared" si="0"/>
+        <v>1.4842664855072356</v>
+      </c>
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v>1.4842664855072356</v>
-      </c>
-      <c r="I10" s="15">
-        <f t="shared" si="2"/>
         <v>7.9242664855072356</v>
       </c>
-      <c r="J10" s="15">
+      <c r="K10" s="15">
         <f>SQRT((2*'SKU Data'!F10*'SKU Data'!J10)/('SKU Data'!D10*'SKU Data'!K10))</f>
         <v>72.777210128237172</v>
       </c>
-      <c r="K10" s="16">
-        <f>IFERROR('SKU Data'!F10/J10,0)</f>
+      <c r="L10" s="16">
+        <f>IFERROR('SKU Data'!F10/K10,0)</f>
         <v>4.5893487729397</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M10" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D10,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f>'SKU Data'!A11</f>
         <v>APP-103</v>
@@ -6394,40 +7545,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A11,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>B</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A11,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>BX</v>
+      </c>
+      <c r="E11" s="14">
         <f>'SKU Data'!G11</f>
         <v>1.17</v>
       </c>
-      <c r="E11" s="14">
+      <c r="F11" s="14">
         <f>'SKU Data'!H11</f>
         <v>0.33</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <f>'SKU Data'!I11</f>
         <v>30</v>
       </c>
-      <c r="G11" s="14">
-        <f t="shared" si="0"/>
+      <c r="H11" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M11,Assumptions!$E$4:$E$6,0))</f>
         <v>1.65</v>
       </c>
-      <c r="H11" s="15">
+      <c r="I11" s="15">
+        <f t="shared" si="0"/>
+        <v>2.9823493256156293</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v>2.9823493256156293</v>
-      </c>
-      <c r="I11" s="15">
-        <f t="shared" si="2"/>
         <v>38.082349325615624</v>
       </c>
-      <c r="J11" s="15">
+      <c r="K11" s="15">
         <f>SQRT((2*'SKU Data'!F11*'SKU Data'!J11)/('SKU Data'!D11*'SKU Data'!K11))</f>
         <v>100.02272469066943</v>
       </c>
-      <c r="K11" s="16">
-        <f>IFERROR('SKU Data'!F11/J11,0)</f>
+      <c r="L11" s="16">
+        <f>IFERROR('SKU Data'!F11/K11,0)</f>
         <v>4.2590321481188278</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M11" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D11,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f>'SKU Data'!A12</f>
         <v>FTW-204</v>
@@ -6440,40 +7599,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A12,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>B</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A12,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>BX</v>
+      </c>
+      <c r="E12" s="14">
         <f>'SKU Data'!G12</f>
         <v>2.33</v>
       </c>
-      <c r="E12" s="14">
+      <c r="F12" s="14">
         <f>'SKU Data'!H12</f>
         <v>1</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <f>'SKU Data'!I12</f>
         <v>45</v>
       </c>
-      <c r="G12" s="14">
-        <f t="shared" si="0"/>
+      <c r="H12" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M12,Assumptions!$E$4:$E$6,0))</f>
         <v>1.65</v>
       </c>
-      <c r="H12" s="15">
+      <c r="I12" s="15">
+        <f t="shared" si="0"/>
+        <v>11.068536488623959</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v>11.068536488623959</v>
-      </c>
-      <c r="I12" s="15">
-        <f t="shared" si="2"/>
         <v>115.91853648862397</v>
       </c>
-      <c r="J12" s="15">
+      <c r="K12" s="15">
         <f>SQRT((2*'SKU Data'!F12*'SKU Data'!J12)/('SKU Data'!D12*'SKU Data'!K12))</f>
         <v>289.66570770842418</v>
       </c>
-      <c r="K12" s="16">
-        <f>IFERROR('SKU Data'!F12/J12,0)</f>
+      <c r="L12" s="16">
+        <f>IFERROR('SKU Data'!F12/K12,0)</f>
         <v>2.9413215901193879</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M12" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D12,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f>'SKU Data'!A13</f>
         <v>HOM-504</v>
@@ -6486,40 +7653,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A13,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>B</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A13,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>BX</v>
+      </c>
+      <c r="E13" s="14">
         <f>'SKU Data'!G13</f>
         <v>2.06</v>
       </c>
-      <c r="E13" s="14">
+      <c r="F13" s="14">
         <f>'SKU Data'!H13</f>
         <v>0.52</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <f>'SKU Data'!I13</f>
         <v>14</v>
       </c>
-      <c r="G13" s="14">
-        <f t="shared" si="0"/>
+      <c r="H13" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M13,Assumptions!$E$4:$E$6,0))</f>
         <v>1.65</v>
       </c>
-      <c r="H13" s="15">
+      <c r="I13" s="15">
+        <f t="shared" si="0"/>
+        <v>3.2103420378520418</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v>3.2103420378520418</v>
-      </c>
-      <c r="I13" s="15">
-        <f t="shared" si="2"/>
         <v>32.05034203785204</v>
       </c>
-      <c r="J13" s="15">
+      <c r="K13" s="15">
         <f>SQRT((2*'SKU Data'!F13*'SKU Data'!J13)/('SKU Data'!D13*'SKU Data'!K13))</f>
         <v>262.83784608258634</v>
       </c>
-      <c r="K13" s="16">
-        <f>IFERROR('SKU Data'!F13/J13,0)</f>
+      <c r="L13" s="16">
+        <f>IFERROR('SKU Data'!F13/K13,0)</f>
         <v>2.861079601769807</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M13" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D13,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f>'SKU Data'!A14</f>
         <v>HOM-501</v>
@@ -6532,40 +7707,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A14,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>B</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A14,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>BX</v>
+      </c>
+      <c r="E14" s="14">
         <f>'SKU Data'!G14</f>
         <v>2.2599999999999998</v>
       </c>
-      <c r="E14" s="14">
+      <c r="F14" s="14">
         <f>'SKU Data'!H14</f>
         <v>0.61</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <f>'SKU Data'!I14</f>
         <v>45</v>
       </c>
-      <c r="G14" s="14">
-        <f t="shared" si="0"/>
+      <c r="H14" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M14,Assumptions!$E$4:$E$6,0))</f>
         <v>1.65</v>
       </c>
-      <c r="H14" s="15">
+      <c r="I14" s="15">
+        <f t="shared" si="0"/>
+        <v>6.751807258060615</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v>6.751807258060615</v>
-      </c>
-      <c r="I14" s="15">
-        <f t="shared" si="2"/>
         <v>108.4518072580606</v>
       </c>
-      <c r="J14" s="15">
+      <c r="K14" s="15">
         <f>SQRT((2*'SKU Data'!F14*'SKU Data'!J14)/('SKU Data'!D14*'SKU Data'!K14))</f>
         <v>302.29059737801617</v>
       </c>
-      <c r="K14" s="16">
-        <f>IFERROR('SKU Data'!F14/J14,0)</f>
+      <c r="L14" s="16">
+        <f>IFERROR('SKU Data'!F14/K14,0)</f>
         <v>2.7291619625480199</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M14" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D14,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f>'SKU Data'!A15</f>
         <v>APP-104</v>
@@ -6578,40 +7761,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A15,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>B</v>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A15,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>BX</v>
+      </c>
+      <c r="E15" s="14">
         <f>'SKU Data'!G15</f>
         <v>0.67</v>
       </c>
-      <c r="E15" s="14">
+      <c r="F15" s="14">
         <f>'SKU Data'!H15</f>
         <v>0.28000000000000003</v>
       </c>
-      <c r="F15">
+      <c r="G15">
         <f>'SKU Data'!I15</f>
         <v>30</v>
       </c>
-      <c r="G15" s="14">
-        <f t="shared" si="0"/>
+      <c r="H15" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M15,Assumptions!$E$4:$E$6,0))</f>
         <v>1.65</v>
       </c>
-      <c r="H15" s="15">
+      <c r="I15" s="15">
+        <f t="shared" si="0"/>
+        <v>2.5304782156738677</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v>2.5304782156738677</v>
-      </c>
-      <c r="I15" s="15">
-        <f t="shared" si="2"/>
         <v>22.630478215673868</v>
       </c>
-      <c r="J15" s="15">
+      <c r="K15" s="15">
         <f>SQRT((2*'SKU Data'!F15*'SKU Data'!J15)/('SKU Data'!D15*'SKU Data'!K15))</f>
         <v>76.443256266144431</v>
       </c>
-      <c r="K15" s="16">
-        <f>IFERROR('SKU Data'!F15/J15,0)</f>
+      <c r="L15" s="16">
+        <f>IFERROR('SKU Data'!F15/K15,0)</f>
         <v>3.1788284783941241</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M15" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D15,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f>'SKU Data'!A16</f>
         <v>ACC-304</v>
@@ -6624,40 +7815,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A16,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>C</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A16,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>CX</v>
+      </c>
+      <c r="E16" s="14">
         <f>'SKU Data'!G16</f>
         <v>2.19</v>
       </c>
-      <c r="E16" s="14">
+      <c r="F16" s="14">
         <f>'SKU Data'!H16</f>
         <v>0.77</v>
       </c>
-      <c r="F16">
+      <c r="G16">
         <f>'SKU Data'!I16</f>
         <v>21</v>
       </c>
-      <c r="G16" s="14">
-        <f t="shared" si="0"/>
+      <c r="H16" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M16,Assumptions!$E$4:$E$6,0))</f>
         <v>1.28</v>
       </c>
-      <c r="H16" s="15">
+      <c r="I16" s="15">
+        <f t="shared" si="0"/>
+        <v>4.5165866049484755</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v>4.5165866049484755</v>
-      </c>
-      <c r="I16" s="15">
-        <f t="shared" si="2"/>
         <v>50.506586604948481</v>
       </c>
-      <c r="J16" s="15">
+      <c r="K16" s="15">
         <f>SQRT((2*'SKU Data'!F16*'SKU Data'!J16)/('SKU Data'!D16*'SKU Data'!K16))</f>
         <v>365.31296886011489</v>
       </c>
-      <c r="K16" s="16">
-        <f>IFERROR('SKU Data'!F16/J16,0)</f>
+      <c r="L16" s="16">
+        <f>IFERROR('SKU Data'!F16/K16,0)</f>
         <v>2.1926404707157214</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M16" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D16,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f>'SKU Data'!A17</f>
         <v>ACC-301</v>
@@ -6670,40 +7869,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A17,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>C</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A17,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>CX</v>
+      </c>
+      <c r="E17" s="14">
         <f>'SKU Data'!G17</f>
         <v>0.94</v>
       </c>
-      <c r="E17" s="14">
+      <c r="F17" s="14">
         <f>'SKU Data'!H17</f>
         <v>0.25</v>
       </c>
-      <c r="F17">
+      <c r="G17">
         <f>'SKU Data'!I17</f>
         <v>21</v>
       </c>
-      <c r="G17" s="14">
-        <f t="shared" si="0"/>
+      <c r="H17" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M17,Assumptions!$E$4:$E$6,0))</f>
         <v>1.28</v>
       </c>
-      <c r="H17" s="15">
+      <c r="I17" s="15">
+        <f t="shared" si="0"/>
+        <v>1.4664242223858688</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v>1.4664242223858688</v>
-      </c>
-      <c r="I17" s="15">
-        <f t="shared" si="2"/>
         <v>21.206424222385866</v>
       </c>
-      <c r="J17" s="15">
+      <c r="K17" s="15">
         <f>SQRT((2*'SKU Data'!F17*'SKU Data'!J17)/('SKU Data'!D17*'SKU Data'!K17))</f>
         <v>153.13760437634471</v>
       </c>
-      <c r="K17" s="16">
-        <f>IFERROR('SKU Data'!F17/J17,0)</f>
+      <c r="L17" s="16">
+        <f>IFERROR('SKU Data'!F17/K17,0)</f>
         <v>2.23981563115652</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M17" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D17,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f>'SKU Data'!A18</f>
         <v>ACC-303</v>
@@ -6716,40 +7923,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A18,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>C</v>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A18,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>CY</v>
+      </c>
+      <c r="E18" s="14">
         <f>'SKU Data'!G18</f>
         <v>0.73</v>
       </c>
-      <c r="E18" s="14">
+      <c r="F18" s="14">
         <f>'SKU Data'!H18</f>
         <v>0.39</v>
       </c>
-      <c r="F18">
+      <c r="G18">
         <f>'SKU Data'!I18</f>
         <v>30</v>
       </c>
-      <c r="G18" s="14">
-        <f t="shared" si="0"/>
+      <c r="H18" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M18,Assumptions!$E$4:$E$6,0))</f>
         <v>1.28</v>
       </c>
-      <c r="H18" s="15">
+      <c r="I18" s="15">
+        <f t="shared" si="0"/>
+        <v>2.7342310070657896</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v>2.7342310070657896</v>
-      </c>
-      <c r="I18" s="15">
-        <f t="shared" si="2"/>
         <v>24.634231007065789</v>
       </c>
-      <c r="J18" s="15">
+      <c r="K18" s="15">
         <f>SQRT((2*'SKU Data'!F18*'SKU Data'!J18)/('SKU Data'!D18*'SKU Data'!K18))</f>
         <v>107.8991904238287</v>
       </c>
-      <c r="K18" s="16">
-        <f>IFERROR('SKU Data'!F18/J18,0)</f>
+      <c r="L18" s="16">
+        <f>IFERROR('SKU Data'!F18/K18,0)</f>
         <v>2.4837999149696519</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M18" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D18,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f>'SKU Data'!A19</f>
         <v>ELE-404</v>
@@ -6762,40 +7977,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A19,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>C</v>
       </c>
-      <c r="D19" s="14">
+      <c r="D19" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A19,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>CX</v>
+      </c>
+      <c r="E19" s="14">
         <f>'SKU Data'!G19</f>
         <v>1.51</v>
       </c>
-      <c r="E19" s="14">
+      <c r="F19" s="14">
         <f>'SKU Data'!H19</f>
         <v>0.48</v>
       </c>
-      <c r="F19">
+      <c r="G19">
         <f>'SKU Data'!I19</f>
         <v>21</v>
       </c>
-      <c r="G19" s="14">
-        <f t="shared" si="0"/>
+      <c r="H19" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M19,Assumptions!$E$4:$E$6,0))</f>
         <v>1.28</v>
       </c>
-      <c r="H19" s="15">
+      <c r="I19" s="15">
+        <f t="shared" si="0"/>
+        <v>2.8155345069808679</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v>2.8155345069808679</v>
-      </c>
-      <c r="I19" s="15">
-        <f t="shared" si="2"/>
         <v>34.525534506980868</v>
       </c>
-      <c r="J19" s="15">
+      <c r="K19" s="15">
         <f>SQRT((2*'SKU Data'!F19*'SKU Data'!J19)/('SKU Data'!D19*'SKU Data'!K19))</f>
         <v>308.27198874957651</v>
       </c>
-      <c r="K19" s="16">
-        <f>IFERROR('SKU Data'!F19/J19,0)</f>
+      <c r="L19" s="16">
+        <f>IFERROR('SKU Data'!F19/K19,0)</f>
         <v>1.7906265250989604</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M19" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D19,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f>'SKU Data'!A20</f>
         <v>HOM-502</v>
@@ -6808,40 +8031,48 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A20,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>C</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A20,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>CY</v>
+      </c>
+      <c r="E20" s="14">
         <f>'SKU Data'!G20</f>
         <v>1.02</v>
       </c>
-      <c r="E20" s="14">
+      <c r="F20" s="14">
         <f>'SKU Data'!H20</f>
         <v>0.52</v>
       </c>
-      <c r="F20">
+      <c r="G20">
         <f>'SKU Data'!I20</f>
         <v>21</v>
       </c>
-      <c r="G20" s="14">
-        <f t="shared" si="0"/>
+      <c r="H20" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M20,Assumptions!$E$4:$E$6,0))</f>
         <v>1.28</v>
       </c>
-      <c r="H20" s="15">
+      <c r="I20" s="15">
+        <f t="shared" si="0"/>
+        <v>3.0501623825626072</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v>3.0501623825626072</v>
-      </c>
-      <c r="I20" s="15">
-        <f t="shared" si="2"/>
         <v>24.470162382562609</v>
       </c>
-      <c r="J20" s="15">
+      <c r="K20" s="15">
         <f>SQRT((2*'SKU Data'!F20*'SKU Data'!J20)/('SKU Data'!D20*'SKU Data'!K20))</f>
         <v>250.09826640171431</v>
       </c>
-      <c r="K20" s="16">
-        <f>IFERROR('SKU Data'!F20/J20,0)</f>
+      <c r="L20" s="16">
+        <f>IFERROR('SKU Data'!F20/K20,0)</f>
         <v>1.4874153481835175</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M20" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D20,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f>'SKU Data'!A21</f>
         <v>APP-102</v>
@@ -6854,41 +8085,96 @@
         <f>INDEX('ABC Analysis'!$H$2:$H$21,MATCH(A21,'ABC Analysis'!$A$2:$A$21,0))</f>
         <v>C</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21" t="str">
+        <f>INDEX('ABC-XYZ Matrix'!$E$2:$E$21,MATCH(A21,'ABC-XYZ Matrix'!$A$2:$A$21,0))</f>
+        <v>CY</v>
+      </c>
+      <c r="E21" s="14">
         <f>'SKU Data'!G21</f>
         <v>0.65</v>
       </c>
-      <c r="E21" s="14">
+      <c r="F21" s="14">
         <f>'SKU Data'!H21</f>
         <v>0.34</v>
       </c>
-      <c r="F21">
+      <c r="G21">
         <f>'SKU Data'!I21</f>
         <v>14</v>
       </c>
-      <c r="G21" s="14">
-        <f t="shared" si="0"/>
+      <c r="H21" s="14">
+        <f>INDEX(Assumptions!$H$4:$H$6,MATCH(M21,Assumptions!$E$4:$E$6,0))</f>
         <v>1.28</v>
       </c>
-      <c r="H21" s="15">
+      <c r="I21" s="15">
+        <f t="shared" si="0"/>
+        <v>1.6283692947240194</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v>1.6283692947240194</v>
-      </c>
-      <c r="I21" s="15">
-        <f t="shared" si="2"/>
         <v>10.728369294724018</v>
       </c>
-      <c r="J21" s="15">
+      <c r="K21" s="15">
         <f>SQRT((2*'SKU Data'!F21*'SKU Data'!J21)/('SKU Data'!D21*'SKU Data'!K21))</f>
         <v>124.29835311089438</v>
       </c>
-      <c r="K21" s="16">
-        <f>IFERROR('SKU Data'!F21/J21,0)</f>
+      <c r="L21" s="16">
+        <f>IFERROR('SKU Data'!F21/K21,0)</f>
         <v>1.9227929736669405</v>
       </c>
+      <c r="M21" s="39">
+        <f>IFERROR(INDEX('Inventory Policy'!$D$4:$D$12,MATCH(D21,'Inventory Policy'!$A$4:$A$12,0)),"Not Found")</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A24" s="51" t="s">
+        <v>170</v>
+      </c>
+      <c r="B24" s="51"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="51"/>
+      <c r="G24" s="51"/>
+      <c r="H24" s="51"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="51"/>
+      <c r="K24" s="51"/>
+    </row>
+    <row r="25" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="B25">
+        <f>COUNTBLANK(H2:H21)</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="53"/>
+      <c r="H25" s="53"/>
+    </row>
+    <row r="26" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B26">
+        <f>COUNTBLANK(I2:I21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B27">
+        <f>COUNTBLANK(J2:J21)</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I21">
+  <mergeCells count="3">
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="A24:D24"/>
+  </mergeCells>
+  <conditionalFormatting sqref="J2:J21">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -6901,6 +8187,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>